<commit_message>
feat(boleto): épico #21 — emissão completa, PDFs, regra delta, multi-perfil
</commit_message>
<xml_diff>
--- a/docs/IMPORTA MAUSER 2 trab.xlsx
+++ b/docs/IMPORTA MAUSER 2 trab.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/23d7ff2762e0afa6/Documentos/Claude/Projects/BSS/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{A630C285-30C7-4CD6-9C51-C6895F52DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9DC4931-C930-4769-A605-66E60092E8D3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{A630C285-30C7-4CD6-9C51-C6895F52DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAE78447-106B-4A30-B903-3BC5A084241A}"/>
   <bookViews>
-    <workbookView xWindow="31560" yWindow="2415" windowWidth="17280" windowHeight="12600" xr2:uid="{153A8857-FD12-4313-8747-6E43C2461CC7}"/>
+    <workbookView xWindow="31455" yWindow="4065" windowWidth="17280" windowHeight="12600" xr2:uid="{153A8857-FD12-4313-8747-6E43C2461CC7}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>CNPJ DA EMPRESA</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>SINDRATEC/RN</t>
-  </si>
-  <si>
-    <t>01.571.635/0002-01</t>
   </si>
 </sst>
 </file>
@@ -135,6 +132,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,15 +449,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C3C62C1-1699-49D6-AECD-B3F0E817624A}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="4" max="4" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -470,7 +471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -484,9 +485,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>7</v>

</xml_diff>